<commit_message>
update GW 32 2025/26
</commit_message>
<xml_diff>
--- a/app/placed_bets.xlsx
+++ b/app/placed_bets.xlsx
@@ -107,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="164">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -581,6 +581,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -963,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T212"/>
+  <dimension ref="A1:T214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1040,7 +1046,7 @@
         </is>
       </c>
       <c r="K1" s="2" t="n"/>
-      <c r="L1" s="162" t="inlineStr">
+      <c r="L1" s="164" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
@@ -1124,38 +1130,38 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J2" s="162" t="n">
+      <c r="J2" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="M2" s="2" t="n">
         <v>55</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>73.93000000000001</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>13410</v>
+        <v>13510</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>12500</v>
+        <v>12613.5</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>-910</v>
+        <v>-896.5</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>-0.88%</t>
+          <t>-0.87%</t>
         </is>
       </c>
       <c r="S2" s="2" t="n">
         <v>1.31</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>120</v>
+        <v>133.5</v>
       </c>
     </row>
     <row r="3">
@@ -1248,7 +1254,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J4" s="162" t="n">
+      <c r="J4" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K4" s="2" t="n"/>
@@ -1300,7 +1306,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J5" s="162" t="n">
+      <c r="J5" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K5" s="2" t="n"/>
@@ -1352,7 +1358,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J6" s="162" t="n">
+      <c r="J6" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K6" s="2" t="n"/>
@@ -1456,7 +1462,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J8" s="162" t="n">
+      <c r="J8" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K8" s="2" t="n"/>
@@ -1560,7 +1566,7 @@
           <t>5 - 1</t>
         </is>
       </c>
-      <c r="J10" s="162" t="n">
+      <c r="J10" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="2" t="n"/>
@@ -1612,7 +1618,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J11" s="162" t="n">
+      <c r="J11" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K11" s="2" t="n"/>
@@ -1716,7 +1722,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J13" s="162" t="n">
+      <c r="J13" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K13" s="2" t="n"/>
@@ -1768,7 +1774,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J14" s="162" t="n">
+      <c r="J14" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K14" s="2" t="n"/>
@@ -1820,7 +1826,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J15" s="162" t="n">
+      <c r="J15" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K15" s="2" t="n"/>
@@ -1872,7 +1878,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J16" s="162" t="n">
+      <c r="J16" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K16" s="2" t="n"/>
@@ -1976,7 +1982,7 @@
           <t>5 - 0</t>
         </is>
       </c>
-      <c r="J18" s="162" t="n">
+      <c r="J18" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="2" t="n"/>
@@ -2080,7 +2086,7 @@
           <t>3 - 3</t>
         </is>
       </c>
-      <c r="J20" s="162" t="n">
+      <c r="J20" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K20" s="2" t="n"/>
@@ -2184,7 +2190,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J22" s="162" t="n">
+      <c r="J22" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K22" s="2" t="n"/>
@@ -2288,7 +2294,7 @@
           <t>4 - 1</t>
         </is>
       </c>
-      <c r="J24" s="162" t="n">
+      <c r="J24" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K24" s="2" t="n"/>
@@ -2340,7 +2346,7 @@
           <t>0 - 6</t>
         </is>
       </c>
-      <c r="J25" s="162" t="n">
+      <c r="J25" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K25" s="2" t="n"/>
@@ -2392,7 +2398,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J26" s="162" t="n">
+      <c r="J26" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K26" s="2" t="n"/>
@@ -2444,7 +2450,7 @@
           <t>4 - 1</t>
         </is>
       </c>
-      <c r="J27" s="162" t="n">
+      <c r="J27" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K27" s="2" t="n"/>
@@ -2496,7 +2502,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J28" s="162" t="n">
+      <c r="J28" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K28" s="2" t="n"/>
@@ -2600,7 +2606,7 @@
           <t>3 - 2</t>
         </is>
       </c>
-      <c r="J30" s="162" t="n">
+      <c r="J30" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K30" s="2" t="n"/>
@@ -2652,7 +2658,7 @@
           <t>0 - 4</t>
         </is>
       </c>
-      <c r="J31" s="162" t="n">
+      <c r="J31" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K31" s="2" t="n"/>
@@ -2704,7 +2710,7 @@
           <t>7 - 1</t>
         </is>
       </c>
-      <c r="J32" s="162" t="n">
+      <c r="J32" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K32" s="2" t="n"/>
@@ -2756,7 +2762,7 @@
           <t>2 - 5</t>
         </is>
       </c>
-      <c r="J33" s="162" t="n">
+      <c r="J33" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K33" s="2" t="n"/>
@@ -2860,7 +2866,7 @@
           <t>4 - 1</t>
         </is>
       </c>
-      <c r="J35" s="162" t="n">
+      <c r="J35" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K35" s="2" t="n"/>
@@ -2912,7 +2918,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J36" s="162" t="n">
+      <c r="J36" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K36" s="2" t="n"/>
@@ -2964,7 +2970,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J37" s="162" t="n">
+      <c r="J37" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K37" s="2" t="n"/>
@@ -3016,7 +3022,7 @@
           <t>3 - 0</t>
         </is>
       </c>
-      <c r="J38" s="162" t="n">
+      <c r="J38" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K38" s="2" t="n"/>
@@ -3068,7 +3074,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J39" s="162" t="n">
+      <c r="J39" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K39" s="2" t="n"/>
@@ -3120,7 +3126,7 @@
           <t>0 - 0</t>
         </is>
       </c>
-      <c r="J40" s="162" t="n">
+      <c r="J40" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K40" s="2" t="n"/>
@@ -3172,7 +3178,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J41" s="162" t="n">
+      <c r="J41" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K41" s="2" t="n"/>
@@ -3224,7 +3230,7 @@
           <t>5 - 1</t>
         </is>
       </c>
-      <c r="J42" s="162" t="n">
+      <c r="J42" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K42" s="2" t="n"/>
@@ -3328,7 +3334,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J44" s="162" t="n">
+      <c r="J44" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K44" s="2" t="n"/>
@@ -3432,7 +3438,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J46" s="162" t="n">
+      <c r="J46" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K46" s="2" t="n"/>
@@ -3484,7 +3490,7 @@
           <t>5 - 1</t>
         </is>
       </c>
-      <c r="J47" s="162" t="n">
+      <c r="J47" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K47" s="2" t="n"/>
@@ -3588,7 +3594,7 @@
           <t>7 - 1</t>
         </is>
       </c>
-      <c r="J49" s="162" t="n">
+      <c r="J49" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K49" s="2" t="n"/>
@@ -3640,7 +3646,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J50" s="162" t="n">
+      <c r="J50" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K50" s="2" t="n"/>
@@ -3692,7 +3698,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J51" s="162" t="n">
+      <c r="J51" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K51" s="2" t="n"/>
@@ -3796,7 +3802,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J53" s="162" t="n">
+      <c r="J53" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K53" s="2" t="n"/>
@@ -3952,7 +3958,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J56" s="162" t="n">
+      <c r="J56" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K56" s="2" t="n"/>
@@ -4004,7 +4010,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J57" s="162" t="n">
+      <c r="J57" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K57" s="2" t="n"/>
@@ -4056,7 +4062,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J58" s="162" t="n">
+      <c r="J58" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K58" s="2" t="n"/>
@@ -4264,7 +4270,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J62" s="162" t="n">
+      <c r="J62" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K62" s="2" t="n"/>
@@ -4316,7 +4322,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J63" s="162" t="n">
+      <c r="J63" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K63" s="2" t="n"/>
@@ -4368,7 +4374,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J64" s="162" t="n">
+      <c r="J64" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K64" s="2" t="n"/>
@@ -4420,7 +4426,7 @@
           <t>3 - 0</t>
         </is>
       </c>
-      <c r="J65" s="162" t="n">
+      <c r="J65" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K65" s="2" t="n"/>
@@ -4524,7 +4530,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J67" s="162" t="n">
+      <c r="J67" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K67" s="2" t="n"/>
@@ -4576,7 +4582,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J68" s="162" t="n">
+      <c r="J68" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K68" s="2" t="n"/>
@@ -4628,7 +4634,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J69" s="162" t="n">
+      <c r="J69" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K69" s="2" t="n"/>
@@ -4680,7 +4686,7 @@
           <t>2 - 3</t>
         </is>
       </c>
-      <c r="J70" s="162" t="n">
+      <c r="J70" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K70" s="2" t="n"/>
@@ -4784,7 +4790,7 @@
           <t>2 - 2</t>
         </is>
       </c>
-      <c r="J72" s="162" t="n">
+      <c r="J72" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K72" s="2" t="n"/>
@@ -4836,7 +4842,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J73" s="162" t="n">
+      <c r="J73" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K73" s="2" t="n"/>
@@ -4888,7 +4894,7 @@
           <t>1 - 4</t>
         </is>
       </c>
-      <c r="J74" s="162" t="n">
+      <c r="J74" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K74" s="2" t="n"/>
@@ -4940,7 +4946,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J75" s="162" t="n">
+      <c r="J75" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K75" s="2" t="n"/>
@@ -4992,7 +4998,7 @@
           <t>3 - 2</t>
         </is>
       </c>
-      <c r="J76" s="162" t="n">
+      <c r="J76" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K76" s="2" t="n"/>
@@ -5148,7 +5154,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J79" s="162" t="n">
+      <c r="J79" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K79" s="2" t="n"/>
@@ -5252,7 +5258,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J81" s="162" t="n">
+      <c r="J81" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K81" s="2" t="n"/>
@@ -5304,7 +5310,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J82" s="162" t="n">
+      <c r="J82" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K82" s="2" t="n"/>
@@ -5460,7 +5466,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J85" s="162" t="n">
+      <c r="J85" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K85" s="2" t="n"/>
@@ -5512,7 +5518,7 @@
           <t>4 - 2</t>
         </is>
       </c>
-      <c r="J86" s="162" t="n">
+      <c r="J86" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K86" s="2" t="n"/>
@@ -5564,7 +5570,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J87" s="162" t="n">
+      <c r="J87" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K87" s="2" t="n"/>
@@ -5616,7 +5622,7 @@
           <t>1 - 3</t>
         </is>
       </c>
-      <c r="J88" s="162" t="n">
+      <c r="J88" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K88" s="2" t="n"/>
@@ -5668,7 +5674,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J89" s="162" t="n">
+      <c r="J89" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K89" s="2" t="n"/>
@@ -5720,7 +5726,7 @@
           <t>1 - 6</t>
         </is>
       </c>
-      <c r="J90" s="162" t="n">
+      <c r="J90" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K90" s="2" t="n"/>
@@ -5772,7 +5778,7 @@
           <t>3 - 2</t>
         </is>
       </c>
-      <c r="J91" s="162" t="n">
+      <c r="J91" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K91" s="2" t="n"/>
@@ -5824,7 +5830,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J92" s="162" t="n">
+      <c r="J92" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K92" s="2" t="n"/>
@@ -5876,7 +5882,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J93" s="162" t="n">
+      <c r="J93" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K93" s="2" t="n"/>
@@ -5928,7 +5934,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J94" s="162" t="n">
+      <c r="J94" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K94" s="2" t="n"/>
@@ -5980,7 +5986,7 @@
           <t>1 - 3</t>
         </is>
       </c>
-      <c r="J95" s="162" t="n">
+      <c r="J95" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K95" s="2" t="n"/>
@@ -6032,7 +6038,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J96" s="162" t="n">
+      <c r="J96" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K96" s="2" t="n"/>
@@ -6084,7 +6090,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J97" s="162" t="n">
+      <c r="J97" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K97" s="2" t="n"/>
@@ -6136,7 +6142,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J98" s="162" t="n">
+      <c r="J98" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K98" s="2" t="n"/>
@@ -6240,7 +6246,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J100" s="162" t="n">
+      <c r="J100" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K100" s="2" t="n"/>
@@ -6292,7 +6298,7 @@
           <t>2 - 2</t>
         </is>
       </c>
-      <c r="J101" s="162" t="n">
+      <c r="J101" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K101" s="2" t="n"/>
@@ -6344,7 +6350,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J102" s="162" t="n">
+      <c r="J102" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K102" s="2" t="n"/>
@@ -6448,7 +6454,7 @@
           <t>5 - 2</t>
         </is>
       </c>
-      <c r="J104" s="162" t="n">
+      <c r="J104" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K104" s="2" t="n"/>
@@ -6500,7 +6506,7 @@
           <t>0 - 0</t>
         </is>
       </c>
-      <c r="J105" s="162" t="n">
+      <c r="J105" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K105" s="2" t="n"/>
@@ -6552,7 +6558,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J106" s="162" t="n">
+      <c r="J106" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K106" s="2" t="n"/>
@@ -6604,7 +6610,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J107" s="162" t="n">
+      <c r="J107" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K107" s="2" t="n"/>
@@ -6656,7 +6662,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J108" s="162" t="n">
+      <c r="J108" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K108" s="2" t="n"/>
@@ -6760,7 +6766,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J110" s="162" t="n">
+      <c r="J110" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K110" s="2" t="n"/>
@@ -6812,7 +6818,7 @@
           <t>3 - 0</t>
         </is>
       </c>
-      <c r="J111" s="162" t="n">
+      <c r="J111" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K111" s="2" t="n"/>
@@ -6864,7 +6870,7 @@
           <t>4 - 2</t>
         </is>
       </c>
-      <c r="J112" s="162" t="n">
+      <c r="J112" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K112" s="2" t="n"/>
@@ -6916,7 +6922,7 @@
           <t>0 - 4</t>
         </is>
       </c>
-      <c r="J113" s="162" t="n">
+      <c r="J113" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K113" s="2" t="n"/>
@@ -6968,7 +6974,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J114" s="162" t="n">
+      <c r="J114" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K114" s="2" t="n"/>
@@ -7020,7 +7026,7 @@
           <t>4 - 3</t>
         </is>
       </c>
-      <c r="J115" s="162" t="n">
+      <c r="J115" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K115" s="2" t="n"/>
@@ -7072,7 +7078,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J116" s="162" t="n">
+      <c r="J116" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K116" s="2" t="n"/>
@@ -7124,7 +7130,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J117" s="162" t="n">
+      <c r="J117" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K117" s="2" t="n"/>
@@ -7176,7 +7182,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J118" s="162" t="n">
+      <c r="J118" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K118" s="2" t="n"/>
@@ -7280,7 +7286,7 @@
           <t>0 - 4</t>
         </is>
       </c>
-      <c r="J120" s="162" t="n">
+      <c r="J120" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K120" s="2" t="n"/>
@@ -7332,7 +7338,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J121" s="162" t="n">
+      <c r="J121" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K121" s="2" t="n"/>
@@ -7436,7 +7442,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J123" s="162" t="n">
+      <c r="J123" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K123" s="2" t="n"/>
@@ -7488,7 +7494,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J124" s="162" t="n">
+      <c r="J124" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K124" s="2" t="n"/>
@@ -7540,7 +7546,7 @@
           <t>2 - 2</t>
         </is>
       </c>
-      <c r="J125" s="162" t="n">
+      <c r="J125" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K125" s="2" t="n"/>
@@ -7644,7 +7650,7 @@
           <t>1 - 3</t>
         </is>
       </c>
-      <c r="J127" s="162" t="n">
+      <c r="J127" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K127" s="2" t="n"/>
@@ -7696,7 +7702,7 @@
           <t>1 - 4</t>
         </is>
       </c>
-      <c r="J128" s="162" t="n">
+      <c r="J128" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K128" s="2" t="n"/>
@@ -7748,7 +7754,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J129" s="162" t="n">
+      <c r="J129" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K129" s="2" t="n"/>
@@ -7852,7 +7858,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J131" s="162" t="n">
+      <c r="J131" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K131" s="2" t="n"/>
@@ -7904,7 +7910,7 @@
           <t>0 - 4</t>
         </is>
       </c>
-      <c r="J132" s="162" t="n">
+      <c r="J132" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K132" s="2" t="n"/>
@@ -7956,7 +7962,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J133" s="162" t="n">
+      <c r="J133" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K133" s="2" t="n"/>
@@ -8008,7 +8014,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J134" s="162" t="n">
+      <c r="J134" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K134" s="2" t="n"/>
@@ -8060,7 +8066,7 @@
           <t>4 - 2</t>
         </is>
       </c>
-      <c r="J135" s="162" t="n">
+      <c r="J135" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K135" s="2" t="n"/>
@@ -8112,7 +8118,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J136" s="162" t="n">
+      <c r="J136" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K136" s="2" t="n"/>
@@ -8164,7 +8170,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J137" s="162" t="n">
+      <c r="J137" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K137" s="2" t="n"/>
@@ -8216,7 +8222,7 @@
           <t>5 - 0</t>
         </is>
       </c>
-      <c r="J138" s="162" t="n">
+      <c r="J138" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K138" s="2" t="n"/>
@@ -8268,7 +8274,7 @@
           <t>2 - 3</t>
         </is>
       </c>
-      <c r="J139" s="162" t="n">
+      <c r="J139" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K139" s="2" t="n"/>
@@ -8320,7 +8326,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J140" s="162" t="n">
+      <c r="J140" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K140" s="2" t="n"/>
@@ -8372,7 +8378,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J141" s="162" t="n">
+      <c r="J141" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K141" s="2" t="n"/>
@@ -8424,7 +8430,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J142" s="162" t="n">
+      <c r="J142" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K142" s="2" t="n"/>
@@ -8528,7 +8534,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J144" s="162" t="n">
+      <c r="J144" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K144" s="2" t="n"/>
@@ -8632,7 +8638,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J146" s="162" t="n">
+      <c r="J146" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K146" s="2" t="n"/>
@@ -8684,7 +8690,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J147" s="162" t="n">
+      <c r="J147" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K147" s="2" t="n"/>
@@ -8736,7 +8742,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J148" s="162" t="n">
+      <c r="J148" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K148" s="2" t="n"/>
@@ -8840,7 +8846,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J150" s="162" t="n">
+      <c r="J150" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K150" s="2" t="n"/>
@@ -8892,7 +8898,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J151" s="162" t="n">
+      <c r="J151" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K151" s="2" t="n"/>
@@ -8944,7 +8950,7 @@
           <t>1 - 4</t>
         </is>
       </c>
-      <c r="J152" s="162" t="n">
+      <c r="J152" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K152" s="2" t="n"/>
@@ -9204,7 +9210,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J157" s="162" t="n">
+      <c r="J157" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K157" s="2" t="n"/>
@@ -9256,7 +9262,7 @@
           <t>5 - 2</t>
         </is>
       </c>
-      <c r="J158" s="162" t="n">
+      <c r="J158" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K158" s="2" t="n"/>
@@ -9308,7 +9314,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J159" s="162" t="n">
+      <c r="J159" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K159" s="2" t="n"/>
@@ -9360,7 +9366,7 @@
           <t>3 - 2</t>
         </is>
       </c>
-      <c r="J160" s="162" t="n">
+      <c r="J160" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K160" s="2" t="n"/>
@@ -9516,7 +9522,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J163" s="162" t="n">
+      <c r="J163" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K163" s="2" t="n"/>
@@ -9568,7 +9574,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J164" s="162" t="n">
+      <c r="J164" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K164" s="2" t="n"/>
@@ -9620,7 +9626,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J165" s="162" t="n">
+      <c r="J165" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K165" s="2" t="n"/>
@@ -9724,7 +9730,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J167" s="162" t="n">
+      <c r="J167" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K167" s="2" t="n"/>
@@ -9828,7 +9834,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J169" s="162" t="n">
+      <c r="J169" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K169" s="2" t="n"/>
@@ -9880,7 +9886,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J170" s="162" t="n">
+      <c r="J170" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K170" s="2" t="n"/>
@@ -9932,7 +9938,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J171" s="162" t="n">
+      <c r="J171" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K171" s="2" t="n"/>
@@ -9984,7 +9990,7 @@
           <t>6 - 2</t>
         </is>
       </c>
-      <c r="J172" s="162" t="n">
+      <c r="J172" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K172" s="2" t="n"/>
@@ -10036,7 +10042,7 @@
           <t>0 - 6</t>
         </is>
       </c>
-      <c r="J173" s="162" t="n">
+      <c r="J173" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K173" s="2" t="n"/>
@@ -10088,7 +10094,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J174" s="162" t="n">
+      <c r="J174" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K174" s="2" t="n"/>
@@ -10192,7 +10198,7 @@
           <t>6 - 1</t>
         </is>
       </c>
-      <c r="J176" s="162" t="n">
+      <c r="J176" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K176" s="2" t="n"/>
@@ -10296,7 +10302,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J178" s="162" t="n">
+      <c r="J178" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K178" s="2" t="n"/>
@@ -10348,7 +10354,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J179" s="162" t="n">
+      <c r="J179" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K179" s="2" t="n"/>
@@ -10400,7 +10406,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J180" s="162" t="n">
+      <c r="J180" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K180" s="2" t="n"/>
@@ -10452,7 +10458,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J181" s="162" t="n">
+      <c r="J181" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K181" s="2" t="n"/>
@@ -10504,7 +10510,7 @@
           <t>6 - 0</t>
         </is>
       </c>
-      <c r="J182" s="162" t="n">
+      <c r="J182" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K182" s="2" t="n"/>
@@ -10608,7 +10614,7 @@
           <t>2 - 4</t>
         </is>
       </c>
-      <c r="J184" s="162" t="n">
+      <c r="J184" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K184" s="2" t="n"/>
@@ -10660,7 +10666,7 @@
           <t>1 - 3</t>
         </is>
       </c>
-      <c r="J185" s="162" t="n">
+      <c r="J185" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K185" s="2" t="n"/>
@@ -10764,7 +10770,7 @@
           <t>3 - 0</t>
         </is>
       </c>
-      <c r="J187" s="162" t="n">
+      <c r="J187" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K187" s="2" t="n"/>
@@ -10868,7 +10874,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J189" s="162" t="n">
+      <c r="J189" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K189" s="2" t="n"/>
@@ -10920,7 +10926,7 @@
           <t>4 - 2</t>
         </is>
       </c>
-      <c r="J190" s="162" t="n">
+      <c r="J190" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K190" s="2" t="n"/>
@@ -11024,7 +11030,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J192" s="162" t="n">
+      <c r="J192" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K192" s="2" t="n"/>
@@ -11076,7 +11082,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J193" s="162" t="n">
+      <c r="J193" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K193" s="2" t="n"/>
@@ -11180,7 +11186,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J195" s="162" t="n">
+      <c r="J195" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K195" s="2" t="n"/>
@@ -11284,7 +11290,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J197" s="162" t="n">
+      <c r="J197" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K197" s="2" t="n"/>
@@ -11336,7 +11342,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J198" s="162" t="n">
+      <c r="J198" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K198" s="2" t="n"/>
@@ -11388,7 +11394,7 @@
           <t>3 - 5</t>
         </is>
       </c>
-      <c r="J199" s="162" t="n">
+      <c r="J199" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K199" s="2" t="n"/>
@@ -11492,7 +11498,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J201" s="162" t="n">
+      <c r="J201" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K201" s="2" t="n"/>
@@ -11544,7 +11550,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J202" s="162" t="n">
+      <c r="J202" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K202" s="2" t="n"/>
@@ -11596,7 +11602,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J203" s="162" t="n">
+      <c r="J203" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K203" s="2" t="n"/>
@@ -11700,7 +11706,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J205" s="162" t="n">
+      <c r="J205" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K205" s="2" t="n"/>
@@ -11752,7 +11758,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J206" s="162" t="n">
+      <c r="J206" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K206" s="2" t="n"/>
@@ -11856,7 +11862,7 @@
           <t>3 - 3</t>
         </is>
       </c>
-      <c r="J208" s="162" t="n">
+      <c r="J208" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K208" s="2" t="n"/>
@@ -11908,7 +11914,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J209" s="162" t="n">
+      <c r="J209" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K209" s="2" t="n"/>
@@ -11960,7 +11966,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J210" s="162" t="n">
+      <c r="J210" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K210" s="2" t="n"/>
@@ -12012,7 +12018,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J211" s="162" t="n">
+      <c r="J211" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K211" s="2" t="n"/>
@@ -12064,7 +12070,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J212" s="162" t="n">
+      <c r="J212" s="164" t="n">
         <v>1</v>
       </c>
       <c r="K212" s="2" t="n"/>
@@ -12077,6 +12083,110 @@
       <c r="R212" s="2" t="n"/>
       <c r="S212" s="2" t="n"/>
       <c r="T212" s="2" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>04.04.2026</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>Bayern Munchen</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="F213" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G213" s="2" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="H213" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>2 - 3</t>
+        </is>
+      </c>
+      <c r="J213" s="164" t="n">
+        <v>1</v>
+      </c>
+      <c r="K213" s="2" t="n"/>
+      <c r="L213" s="2" t="n"/>
+      <c r="M213" s="2" t="n"/>
+      <c r="N213" s="2" t="n"/>
+      <c r="O213" s="2" t="n"/>
+      <c r="P213" s="2" t="n"/>
+      <c r="Q213" s="2" t="n"/>
+      <c r="R213" s="2" t="n"/>
+      <c r="S213" s="2" t="n"/>
+      <c r="T213" s="2" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>11.04.2026</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>St.Pauli</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>Bayern Munchen</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F214" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G214" s="2" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="H214" s="2" t="n">
+        <v>5.000000000000007</v>
+      </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>0 - 5</t>
+        </is>
+      </c>
+      <c r="J214" s="164" t="n">
+        <v>1</v>
+      </c>
+      <c r="K214" s="2" t="n"/>
+      <c r="L214" s="2" t="n"/>
+      <c r="M214" s="2" t="n"/>
+      <c r="N214" s="2" t="n"/>
+      <c r="O214" s="2" t="n"/>
+      <c r="P214" s="2" t="n"/>
+      <c r="Q214" s="2" t="n"/>
+      <c r="R214" s="2" t="n"/>
+      <c r="S214" s="2" t="n"/>
+      <c r="T214" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12289,14 +12399,14 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>90.0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update GW 35 2025/26
</commit_message>
<xml_diff>
--- a/app/placed_bets.xlsx
+++ b/app/placed_bets.xlsx
@@ -107,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -602,6 +602,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -969,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T214"/>
+  <dimension ref="A1:T216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1046,7 +1052,7 @@
         </is>
       </c>
       <c r="K1" s="2" t="n"/>
-      <c r="L1" s="164" t="inlineStr">
+      <c r="L1" s="165" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
@@ -1130,38 +1136,38 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J2" s="164" t="n">
+      <c r="J2" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>74.18000000000001</v>
+        <v>73.95</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>13510</v>
+        <v>13610</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>12613.5</v>
+        <v>12672</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>-896.5</v>
+        <v>-938</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>-0.87%</t>
+          <t>-0.91%</t>
         </is>
       </c>
       <c r="S2" s="2" t="n">
         <v>1.31</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>133.5</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -1254,7 +1260,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J4" s="164" t="n">
+      <c r="J4" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K4" s="2" t="n"/>
@@ -1306,7 +1312,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J5" s="164" t="n">
+      <c r="J5" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K5" s="2" t="n"/>
@@ -1358,7 +1364,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J6" s="164" t="n">
+      <c r="J6" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K6" s="2" t="n"/>
@@ -1462,7 +1468,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J8" s="164" t="n">
+      <c r="J8" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K8" s="2" t="n"/>
@@ -1566,7 +1572,7 @@
           <t>5 - 1</t>
         </is>
       </c>
-      <c r="J10" s="164" t="n">
+      <c r="J10" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="2" t="n"/>
@@ -1618,7 +1624,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J11" s="164" t="n">
+      <c r="J11" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K11" s="2" t="n"/>
@@ -1722,7 +1728,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J13" s="164" t="n">
+      <c r="J13" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K13" s="2" t="n"/>
@@ -1774,7 +1780,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J14" s="164" t="n">
+      <c r="J14" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K14" s="2" t="n"/>
@@ -1826,7 +1832,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J15" s="164" t="n">
+      <c r="J15" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K15" s="2" t="n"/>
@@ -1878,7 +1884,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J16" s="164" t="n">
+      <c r="J16" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K16" s="2" t="n"/>
@@ -1982,7 +1988,7 @@
           <t>5 - 0</t>
         </is>
       </c>
-      <c r="J18" s="164" t="n">
+      <c r="J18" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="2" t="n"/>
@@ -2086,7 +2092,7 @@
           <t>3 - 3</t>
         </is>
       </c>
-      <c r="J20" s="164" t="n">
+      <c r="J20" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K20" s="2" t="n"/>
@@ -2190,7 +2196,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J22" s="164" t="n">
+      <c r="J22" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K22" s="2" t="n"/>
@@ -2294,7 +2300,7 @@
           <t>4 - 1</t>
         </is>
       </c>
-      <c r="J24" s="164" t="n">
+      <c r="J24" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K24" s="2" t="n"/>
@@ -2346,7 +2352,7 @@
           <t>0 - 6</t>
         </is>
       </c>
-      <c r="J25" s="164" t="n">
+      <c r="J25" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K25" s="2" t="n"/>
@@ -2398,7 +2404,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J26" s="164" t="n">
+      <c r="J26" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K26" s="2" t="n"/>
@@ -2450,7 +2456,7 @@
           <t>4 - 1</t>
         </is>
       </c>
-      <c r="J27" s="164" t="n">
+      <c r="J27" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K27" s="2" t="n"/>
@@ -2502,7 +2508,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J28" s="164" t="n">
+      <c r="J28" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K28" s="2" t="n"/>
@@ -2606,7 +2612,7 @@
           <t>3 - 2</t>
         </is>
       </c>
-      <c r="J30" s="164" t="n">
+      <c r="J30" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K30" s="2" t="n"/>
@@ -2658,7 +2664,7 @@
           <t>0 - 4</t>
         </is>
       </c>
-      <c r="J31" s="164" t="n">
+      <c r="J31" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K31" s="2" t="n"/>
@@ -2710,7 +2716,7 @@
           <t>7 - 1</t>
         </is>
       </c>
-      <c r="J32" s="164" t="n">
+      <c r="J32" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K32" s="2" t="n"/>
@@ -2762,7 +2768,7 @@
           <t>2 - 5</t>
         </is>
       </c>
-      <c r="J33" s="164" t="n">
+      <c r="J33" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K33" s="2" t="n"/>
@@ -2866,7 +2872,7 @@
           <t>4 - 1</t>
         </is>
       </c>
-      <c r="J35" s="164" t="n">
+      <c r="J35" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K35" s="2" t="n"/>
@@ -2918,7 +2924,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J36" s="164" t="n">
+      <c r="J36" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K36" s="2" t="n"/>
@@ -2970,7 +2976,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J37" s="164" t="n">
+      <c r="J37" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K37" s="2" t="n"/>
@@ -3022,7 +3028,7 @@
           <t>3 - 0</t>
         </is>
       </c>
-      <c r="J38" s="164" t="n">
+      <c r="J38" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K38" s="2" t="n"/>
@@ -3074,7 +3080,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J39" s="164" t="n">
+      <c r="J39" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K39" s="2" t="n"/>
@@ -3126,7 +3132,7 @@
           <t>0 - 0</t>
         </is>
       </c>
-      <c r="J40" s="164" t="n">
+      <c r="J40" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K40" s="2" t="n"/>
@@ -3178,7 +3184,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J41" s="164" t="n">
+      <c r="J41" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K41" s="2" t="n"/>
@@ -3230,7 +3236,7 @@
           <t>5 - 1</t>
         </is>
       </c>
-      <c r="J42" s="164" t="n">
+      <c r="J42" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K42" s="2" t="n"/>
@@ -3334,7 +3340,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J44" s="164" t="n">
+      <c r="J44" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K44" s="2" t="n"/>
@@ -3438,7 +3444,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J46" s="164" t="n">
+      <c r="J46" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K46" s="2" t="n"/>
@@ -3490,7 +3496,7 @@
           <t>5 - 1</t>
         </is>
       </c>
-      <c r="J47" s="164" t="n">
+      <c r="J47" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K47" s="2" t="n"/>
@@ -3594,7 +3600,7 @@
           <t>7 - 1</t>
         </is>
       </c>
-      <c r="J49" s="164" t="n">
+      <c r="J49" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K49" s="2" t="n"/>
@@ -3646,7 +3652,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J50" s="164" t="n">
+      <c r="J50" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K50" s="2" t="n"/>
@@ -3698,7 +3704,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J51" s="164" t="n">
+      <c r="J51" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K51" s="2" t="n"/>
@@ -3802,7 +3808,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J53" s="164" t="n">
+      <c r="J53" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K53" s="2" t="n"/>
@@ -3958,7 +3964,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J56" s="164" t="n">
+      <c r="J56" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K56" s="2" t="n"/>
@@ -4010,7 +4016,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J57" s="164" t="n">
+      <c r="J57" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K57" s="2" t="n"/>
@@ -4062,7 +4068,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J58" s="164" t="n">
+      <c r="J58" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K58" s="2" t="n"/>
@@ -4270,7 +4276,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J62" s="164" t="n">
+      <c r="J62" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K62" s="2" t="n"/>
@@ -4322,7 +4328,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J63" s="164" t="n">
+      <c r="J63" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K63" s="2" t="n"/>
@@ -4374,7 +4380,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J64" s="164" t="n">
+      <c r="J64" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K64" s="2" t="n"/>
@@ -4426,7 +4432,7 @@
           <t>3 - 0</t>
         </is>
       </c>
-      <c r="J65" s="164" t="n">
+      <c r="J65" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K65" s="2" t="n"/>
@@ -4530,7 +4536,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J67" s="164" t="n">
+      <c r="J67" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K67" s="2" t="n"/>
@@ -4582,7 +4588,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J68" s="164" t="n">
+      <c r="J68" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K68" s="2" t="n"/>
@@ -4634,7 +4640,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J69" s="164" t="n">
+      <c r="J69" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K69" s="2" t="n"/>
@@ -4686,7 +4692,7 @@
           <t>2 - 3</t>
         </is>
       </c>
-      <c r="J70" s="164" t="n">
+      <c r="J70" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K70" s="2" t="n"/>
@@ -4790,7 +4796,7 @@
           <t>2 - 2</t>
         </is>
       </c>
-      <c r="J72" s="164" t="n">
+      <c r="J72" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K72" s="2" t="n"/>
@@ -4842,7 +4848,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J73" s="164" t="n">
+      <c r="J73" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K73" s="2" t="n"/>
@@ -4894,7 +4900,7 @@
           <t>1 - 4</t>
         </is>
       </c>
-      <c r="J74" s="164" t="n">
+      <c r="J74" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K74" s="2" t="n"/>
@@ -4946,7 +4952,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J75" s="164" t="n">
+      <c r="J75" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K75" s="2" t="n"/>
@@ -4998,7 +5004,7 @@
           <t>3 - 2</t>
         </is>
       </c>
-      <c r="J76" s="164" t="n">
+      <c r="J76" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K76" s="2" t="n"/>
@@ -5154,7 +5160,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J79" s="164" t="n">
+      <c r="J79" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K79" s="2" t="n"/>
@@ -5258,7 +5264,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J81" s="164" t="n">
+      <c r="J81" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K81" s="2" t="n"/>
@@ -5310,7 +5316,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J82" s="164" t="n">
+      <c r="J82" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K82" s="2" t="n"/>
@@ -5466,7 +5472,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J85" s="164" t="n">
+      <c r="J85" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K85" s="2" t="n"/>
@@ -5518,7 +5524,7 @@
           <t>4 - 2</t>
         </is>
       </c>
-      <c r="J86" s="164" t="n">
+      <c r="J86" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K86" s="2" t="n"/>
@@ -5570,7 +5576,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J87" s="164" t="n">
+      <c r="J87" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K87" s="2" t="n"/>
@@ -5622,7 +5628,7 @@
           <t>1 - 3</t>
         </is>
       </c>
-      <c r="J88" s="164" t="n">
+      <c r="J88" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K88" s="2" t="n"/>
@@ -5674,7 +5680,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J89" s="164" t="n">
+      <c r="J89" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K89" s="2" t="n"/>
@@ -5726,7 +5732,7 @@
           <t>1 - 6</t>
         </is>
       </c>
-      <c r="J90" s="164" t="n">
+      <c r="J90" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K90" s="2" t="n"/>
@@ -5778,7 +5784,7 @@
           <t>3 - 2</t>
         </is>
       </c>
-      <c r="J91" s="164" t="n">
+      <c r="J91" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K91" s="2" t="n"/>
@@ -5830,7 +5836,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J92" s="164" t="n">
+      <c r="J92" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K92" s="2" t="n"/>
@@ -5882,7 +5888,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J93" s="164" t="n">
+      <c r="J93" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K93" s="2" t="n"/>
@@ -5934,7 +5940,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J94" s="164" t="n">
+      <c r="J94" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K94" s="2" t="n"/>
@@ -5986,7 +5992,7 @@
           <t>1 - 3</t>
         </is>
       </c>
-      <c r="J95" s="164" t="n">
+      <c r="J95" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K95" s="2" t="n"/>
@@ -6038,7 +6044,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J96" s="164" t="n">
+      <c r="J96" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K96" s="2" t="n"/>
@@ -6090,7 +6096,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J97" s="164" t="n">
+      <c r="J97" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K97" s="2" t="n"/>
@@ -6142,7 +6148,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J98" s="164" t="n">
+      <c r="J98" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K98" s="2" t="n"/>
@@ -6246,7 +6252,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J100" s="164" t="n">
+      <c r="J100" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K100" s="2" t="n"/>
@@ -6298,7 +6304,7 @@
           <t>2 - 2</t>
         </is>
       </c>
-      <c r="J101" s="164" t="n">
+      <c r="J101" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K101" s="2" t="n"/>
@@ -6350,7 +6356,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J102" s="164" t="n">
+      <c r="J102" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K102" s="2" t="n"/>
@@ -6454,7 +6460,7 @@
           <t>5 - 2</t>
         </is>
       </c>
-      <c r="J104" s="164" t="n">
+      <c r="J104" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K104" s="2" t="n"/>
@@ -6506,7 +6512,7 @@
           <t>0 - 0</t>
         </is>
       </c>
-      <c r="J105" s="164" t="n">
+      <c r="J105" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K105" s="2" t="n"/>
@@ -6558,7 +6564,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J106" s="164" t="n">
+      <c r="J106" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K106" s="2" t="n"/>
@@ -6610,7 +6616,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J107" s="164" t="n">
+      <c r="J107" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K107" s="2" t="n"/>
@@ -6662,7 +6668,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J108" s="164" t="n">
+      <c r="J108" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K108" s="2" t="n"/>
@@ -6766,7 +6772,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J110" s="164" t="n">
+      <c r="J110" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K110" s="2" t="n"/>
@@ -6818,7 +6824,7 @@
           <t>3 - 0</t>
         </is>
       </c>
-      <c r="J111" s="164" t="n">
+      <c r="J111" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K111" s="2" t="n"/>
@@ -6870,7 +6876,7 @@
           <t>4 - 2</t>
         </is>
       </c>
-      <c r="J112" s="164" t="n">
+      <c r="J112" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K112" s="2" t="n"/>
@@ -6922,7 +6928,7 @@
           <t>0 - 4</t>
         </is>
       </c>
-      <c r="J113" s="164" t="n">
+      <c r="J113" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K113" s="2" t="n"/>
@@ -6974,7 +6980,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J114" s="164" t="n">
+      <c r="J114" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K114" s="2" t="n"/>
@@ -7026,7 +7032,7 @@
           <t>4 - 3</t>
         </is>
       </c>
-      <c r="J115" s="164" t="n">
+      <c r="J115" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K115" s="2" t="n"/>
@@ -7078,7 +7084,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J116" s="164" t="n">
+      <c r="J116" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K116" s="2" t="n"/>
@@ -7130,7 +7136,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J117" s="164" t="n">
+      <c r="J117" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K117" s="2" t="n"/>
@@ -7182,7 +7188,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J118" s="164" t="n">
+      <c r="J118" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K118" s="2" t="n"/>
@@ -7286,7 +7292,7 @@
           <t>0 - 4</t>
         </is>
       </c>
-      <c r="J120" s="164" t="n">
+      <c r="J120" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K120" s="2" t="n"/>
@@ -7338,7 +7344,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J121" s="164" t="n">
+      <c r="J121" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K121" s="2" t="n"/>
@@ -7442,7 +7448,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J123" s="164" t="n">
+      <c r="J123" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K123" s="2" t="n"/>
@@ -7494,7 +7500,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J124" s="164" t="n">
+      <c r="J124" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K124" s="2" t="n"/>
@@ -7546,7 +7552,7 @@
           <t>2 - 2</t>
         </is>
       </c>
-      <c r="J125" s="164" t="n">
+      <c r="J125" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K125" s="2" t="n"/>
@@ -7650,7 +7656,7 @@
           <t>1 - 3</t>
         </is>
       </c>
-      <c r="J127" s="164" t="n">
+      <c r="J127" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K127" s="2" t="n"/>
@@ -7702,7 +7708,7 @@
           <t>1 - 4</t>
         </is>
       </c>
-      <c r="J128" s="164" t="n">
+      <c r="J128" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K128" s="2" t="n"/>
@@ -7754,7 +7760,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J129" s="164" t="n">
+      <c r="J129" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K129" s="2" t="n"/>
@@ -7858,7 +7864,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J131" s="164" t="n">
+      <c r="J131" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K131" s="2" t="n"/>
@@ -7910,7 +7916,7 @@
           <t>0 - 4</t>
         </is>
       </c>
-      <c r="J132" s="164" t="n">
+      <c r="J132" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K132" s="2" t="n"/>
@@ -7962,7 +7968,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J133" s="164" t="n">
+      <c r="J133" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K133" s="2" t="n"/>
@@ -8014,7 +8020,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J134" s="164" t="n">
+      <c r="J134" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K134" s="2" t="n"/>
@@ -8066,7 +8072,7 @@
           <t>4 - 2</t>
         </is>
       </c>
-      <c r="J135" s="164" t="n">
+      <c r="J135" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K135" s="2" t="n"/>
@@ -8118,7 +8124,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J136" s="164" t="n">
+      <c r="J136" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K136" s="2" t="n"/>
@@ -8170,7 +8176,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J137" s="164" t="n">
+      <c r="J137" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K137" s="2" t="n"/>
@@ -8222,7 +8228,7 @@
           <t>5 - 0</t>
         </is>
       </c>
-      <c r="J138" s="164" t="n">
+      <c r="J138" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K138" s="2" t="n"/>
@@ -8274,7 +8280,7 @@
           <t>2 - 3</t>
         </is>
       </c>
-      <c r="J139" s="164" t="n">
+      <c r="J139" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K139" s="2" t="n"/>
@@ -8326,7 +8332,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J140" s="164" t="n">
+      <c r="J140" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K140" s="2" t="n"/>
@@ -8378,7 +8384,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J141" s="164" t="n">
+      <c r="J141" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K141" s="2" t="n"/>
@@ -8430,7 +8436,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J142" s="164" t="n">
+      <c r="J142" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K142" s="2" t="n"/>
@@ -8534,7 +8540,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J144" s="164" t="n">
+      <c r="J144" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K144" s="2" t="n"/>
@@ -8638,7 +8644,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J146" s="164" t="n">
+      <c r="J146" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K146" s="2" t="n"/>
@@ -8690,7 +8696,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J147" s="164" t="n">
+      <c r="J147" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K147" s="2" t="n"/>
@@ -8742,7 +8748,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J148" s="164" t="n">
+      <c r="J148" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K148" s="2" t="n"/>
@@ -8846,7 +8852,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J150" s="164" t="n">
+      <c r="J150" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K150" s="2" t="n"/>
@@ -8898,7 +8904,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J151" s="164" t="n">
+      <c r="J151" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K151" s="2" t="n"/>
@@ -8950,7 +8956,7 @@
           <t>1 - 4</t>
         </is>
       </c>
-      <c r="J152" s="164" t="n">
+      <c r="J152" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K152" s="2" t="n"/>
@@ -9210,7 +9216,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J157" s="164" t="n">
+      <c r="J157" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K157" s="2" t="n"/>
@@ -9262,7 +9268,7 @@
           <t>5 - 2</t>
         </is>
       </c>
-      <c r="J158" s="164" t="n">
+      <c r="J158" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K158" s="2" t="n"/>
@@ -9314,7 +9320,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J159" s="164" t="n">
+      <c r="J159" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K159" s="2" t="n"/>
@@ -9366,7 +9372,7 @@
           <t>3 - 2</t>
         </is>
       </c>
-      <c r="J160" s="164" t="n">
+      <c r="J160" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K160" s="2" t="n"/>
@@ -9522,7 +9528,7 @@
           <t>0 - 2</t>
         </is>
       </c>
-      <c r="J163" s="164" t="n">
+      <c r="J163" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K163" s="2" t="n"/>
@@ -9574,7 +9580,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J164" s="164" t="n">
+      <c r="J164" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K164" s="2" t="n"/>
@@ -9626,7 +9632,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J165" s="164" t="n">
+      <c r="J165" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K165" s="2" t="n"/>
@@ -9730,7 +9736,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J167" s="164" t="n">
+      <c r="J167" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K167" s="2" t="n"/>
@@ -9834,7 +9840,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J169" s="164" t="n">
+      <c r="J169" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K169" s="2" t="n"/>
@@ -9886,7 +9892,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J170" s="164" t="n">
+      <c r="J170" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K170" s="2" t="n"/>
@@ -9938,7 +9944,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J171" s="164" t="n">
+      <c r="J171" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K171" s="2" t="n"/>
@@ -9990,7 +9996,7 @@
           <t>6 - 2</t>
         </is>
       </c>
-      <c r="J172" s="164" t="n">
+      <c r="J172" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K172" s="2" t="n"/>
@@ -10042,7 +10048,7 @@
           <t>0 - 6</t>
         </is>
       </c>
-      <c r="J173" s="164" t="n">
+      <c r="J173" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K173" s="2" t="n"/>
@@ -10094,7 +10100,7 @@
           <t>0 - 3</t>
         </is>
       </c>
-      <c r="J174" s="164" t="n">
+      <c r="J174" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K174" s="2" t="n"/>
@@ -10198,7 +10204,7 @@
           <t>6 - 1</t>
         </is>
       </c>
-      <c r="J176" s="164" t="n">
+      <c r="J176" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K176" s="2" t="n"/>
@@ -10302,7 +10308,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J178" s="164" t="n">
+      <c r="J178" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K178" s="2" t="n"/>
@@ -10354,7 +10360,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J179" s="164" t="n">
+      <c r="J179" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K179" s="2" t="n"/>
@@ -10406,7 +10412,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J180" s="164" t="n">
+      <c r="J180" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K180" s="2" t="n"/>
@@ -10458,7 +10464,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J181" s="164" t="n">
+      <c r="J181" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K181" s="2" t="n"/>
@@ -10510,7 +10516,7 @@
           <t>6 - 0</t>
         </is>
       </c>
-      <c r="J182" s="164" t="n">
+      <c r="J182" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K182" s="2" t="n"/>
@@ -10614,7 +10620,7 @@
           <t>2 - 4</t>
         </is>
       </c>
-      <c r="J184" s="164" t="n">
+      <c r="J184" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K184" s="2" t="n"/>
@@ -10666,7 +10672,7 @@
           <t>1 - 3</t>
         </is>
       </c>
-      <c r="J185" s="164" t="n">
+      <c r="J185" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K185" s="2" t="n"/>
@@ -10770,7 +10776,7 @@
           <t>3 - 0</t>
         </is>
       </c>
-      <c r="J187" s="164" t="n">
+      <c r="J187" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K187" s="2" t="n"/>
@@ -10874,7 +10880,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J189" s="164" t="n">
+      <c r="J189" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K189" s="2" t="n"/>
@@ -10926,7 +10932,7 @@
           <t>4 - 2</t>
         </is>
       </c>
-      <c r="J190" s="164" t="n">
+      <c r="J190" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K190" s="2" t="n"/>
@@ -11030,7 +11036,7 @@
           <t>3 - 1</t>
         </is>
       </c>
-      <c r="J192" s="164" t="n">
+      <c r="J192" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K192" s="2" t="n"/>
@@ -11082,7 +11088,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J193" s="164" t="n">
+      <c r="J193" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K193" s="2" t="n"/>
@@ -11186,7 +11192,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J195" s="164" t="n">
+      <c r="J195" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K195" s="2" t="n"/>
@@ -11290,7 +11296,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J197" s="164" t="n">
+      <c r="J197" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K197" s="2" t="n"/>
@@ -11342,7 +11348,7 @@
           <t>1 - 1</t>
         </is>
       </c>
-      <c r="J198" s="164" t="n">
+      <c r="J198" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K198" s="2" t="n"/>
@@ -11394,7 +11400,7 @@
           <t>3 - 5</t>
         </is>
       </c>
-      <c r="J199" s="164" t="n">
+      <c r="J199" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K199" s="2" t="n"/>
@@ -11498,7 +11504,7 @@
           <t>2 - 1</t>
         </is>
       </c>
-      <c r="J201" s="164" t="n">
+      <c r="J201" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K201" s="2" t="n"/>
@@ -11550,7 +11556,7 @@
           <t>2 - 0</t>
         </is>
       </c>
-      <c r="J202" s="164" t="n">
+      <c r="J202" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K202" s="2" t="n"/>
@@ -11602,7 +11608,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J203" s="164" t="n">
+      <c r="J203" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K203" s="2" t="n"/>
@@ -11706,7 +11712,7 @@
           <t>1 - 2</t>
         </is>
       </c>
-      <c r="J205" s="164" t="n">
+      <c r="J205" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K205" s="2" t="n"/>
@@ -11758,7 +11764,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J206" s="164" t="n">
+      <c r="J206" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K206" s="2" t="n"/>
@@ -11862,7 +11868,7 @@
           <t>3 - 3</t>
         </is>
       </c>
-      <c r="J208" s="164" t="n">
+      <c r="J208" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K208" s="2" t="n"/>
@@ -11914,7 +11920,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J209" s="164" t="n">
+      <c r="J209" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K209" s="2" t="n"/>
@@ -11966,7 +11972,7 @@
           <t>0 - 1</t>
         </is>
       </c>
-      <c r="J210" s="164" t="n">
+      <c r="J210" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K210" s="2" t="n"/>
@@ -12018,7 +12024,7 @@
           <t>4 - 0</t>
         </is>
       </c>
-      <c r="J211" s="164" t="n">
+      <c r="J211" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K211" s="2" t="n"/>
@@ -12070,7 +12076,7 @@
           <t>1 - 0</t>
         </is>
       </c>
-      <c r="J212" s="164" t="n">
+      <c r="J212" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K212" s="2" t="n"/>
@@ -12122,7 +12128,7 @@
           <t>2 - 3</t>
         </is>
       </c>
-      <c r="J213" s="164" t="n">
+      <c r="J213" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K213" s="2" t="n"/>
@@ -12174,7 +12180,7 @@
           <t>0 - 5</t>
         </is>
       </c>
-      <c r="J214" s="164" t="n">
+      <c r="J214" s="165" t="n">
         <v>1</v>
       </c>
       <c r="K214" s="2" t="n"/>
@@ -12187,6 +12193,110 @@
       <c r="R214" s="2" t="n"/>
       <c r="S214" s="2" t="n"/>
       <c r="T214" s="2" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>Olympique Lyon</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>Auxerre</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="F215" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G215" s="2" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="H215" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>3 - 2</t>
+        </is>
+      </c>
+      <c r="J215" s="165" t="n">
+        <v>1</v>
+      </c>
+      <c r="K215" s="2" t="n"/>
+      <c r="L215" s="2" t="n"/>
+      <c r="M215" s="2" t="n"/>
+      <c r="N215" s="2" t="n"/>
+      <c r="O215" s="2" t="n"/>
+      <c r="P215" s="2" t="n"/>
+      <c r="Q215" s="2" t="n"/>
+      <c r="R215" s="2" t="n"/>
+      <c r="S215" s="2" t="n"/>
+      <c r="T215" s="2" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>02.05.2026</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Bayern Munchen</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>Heidenheim</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F216" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G216" s="2" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="H216" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>3 - 3</t>
+        </is>
+      </c>
+      <c r="J216" s="158" t="n">
+        <v>0</v>
+      </c>
+      <c r="K216" s="2" t="n"/>
+      <c r="L216" s="2" t="n"/>
+      <c r="M216" s="2" t="n"/>
+      <c r="N216" s="2" t="n"/>
+      <c r="O216" s="2" t="n"/>
+      <c r="P216" s="2" t="n"/>
+      <c r="Q216" s="2" t="n"/>
+      <c r="R216" s="2" t="n"/>
+      <c r="S216" s="2" t="n"/>
+      <c r="T216" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12399,14 +12509,14 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>9</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>81.82%</t>
         </is>
       </c>
     </row>
@@ -12633,14 +12743,14 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>

</xml_diff>